<commit_message>
Modificacion y mejora de las actividades
</commit_message>
<xml_diff>
--- a/Actividades/actividades.xlsx
+++ b/Actividades/actividades.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>USUARIO</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -470,6 +470,1431 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>OBSERVACIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-03-09 10:40:34</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>BIBLIOTECAS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Saudith</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>LLAMADA TELEFONICA</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Se solicita la visita y solicitud a la biblioteca para la revision de la intermitencia del internet, se radica la solicitud a tigo une</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Se solicita la visita y solicitud a la biblioteca para la revision de la intermitencia del internet, se radica la solicitud a tigo une</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-03-09 10:49:07</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Elizabeth</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se solicita la asignación de permisos a un funcionario nuevo, se hace la asignación de permisos pertinente, se le informa a la solicitante la asignación de estos permisos </t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se solicita la asignación de permisos a un funcionario nuevo, se hace la asignación de permisos pertinente, se le informa a la solicitante la asignación de estos permisos </t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>6.	Apoyar en la documentación técnica del área, incluyendo la organización y archivo de documentos, informes de soporte y demás registros, de acuerdo con las directrices internas y del Sistema de Gestión de Calidad.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-03-09 10:52:03</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ARCHIVO GENERAL</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Edwin</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos necesarios para continuar con la función y son necesario para el solicitante, se asignan los permisos solicitados y se le informa al solicitante</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos necesarios para continuar con la función y son necesario para el solicitante, se asignan los permisos solicitados y se le informa al solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>6.	Apoyar en la documentación técnica del área, incluyendo la organización y archivo de documentos, informes de soporte y demás registros, de acuerdo con las directrices internas y del Sistema de Gestión de Calidad.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-03-09 11:24:20</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CATASTRO</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se solicita la creación y asignación de permisos a un nuevo funcionario, se hace los requerimientos solicitados y se le informan a la solicitante </t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se solicita la creación y asignación de permisos a un nuevo funcionario, se hace los requerimientos solicitados y se le informan a la solicitante </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>6.	Apoyar en la documentación técnica del área, incluyendo la organización y archivo de documentos, informes de soporte y demás registros, de acuerdo con las directrices internas y del Sistema de Gestión de Calidad.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-03-10 15:11:18</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Elizabeth</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos a un funcionario, se asignan los permisos solicitados y se le informa a la solicitante</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos a un funcionario, se asignan los permisos solicitados y se le informa a la solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>4.	Apoyar en tareas logísticas relacionadas con la infraestructura tecnológica, tales como instalación, traslado o reubicación de equipos de cómputo, dispositivos de red y demás componentes tecnológicos, bajo supervisión del personal del área.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-03-11 15:12:49</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>INFRAESTRUCTURA</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación de nueva impresora en la oficina de Familia, se hace la instalación respectiva y se evidencia el funcionamiento de la impresora</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación de nueva impresora en la oficina de Familia, se hace la instalación respectiva y se evidencia el funcionamiento de la impresora</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-03-10 15:20:23</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>FAMILIA</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación de la impresora en el equipo, se hace la instalación respectiva y se le evidencia a la solicitante</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación de la impresora en el equipo, se hace la instalación respectiva y se le evidencia a la solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-03-10 15:22:53</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FAMILIA</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación del escáner en el equipo, se hace la instalación con permiso del jefe inmediado de la solicitante y se evidencia la solicitante</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación del escáner en el equipo, se hace la instalación con permiso del jefe inmediado de la solicitante y se evidencia la solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-03-10 15:24:18</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>FAMILIA</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Patricia</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se solicita la instalación del escáner con permiso del jefe inmediato de la solicitante, se hace la instalación respectiva y se le evidencia el funcionamiento </t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se solicita la instalación del escáner con permiso del jefe inmediato de la solicitante, se hace la instalación respectiva y se le evidencia el funcionamiento </t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>4.	Apoyar en tareas logísticas relacionadas con la infraestructura tecnológica, tales como instalación, traslado o reubicación de equipos de cómputo, dispositivos de red y demás componentes tecnológicos, bajo supervisión del personal del área.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-03-10 08:12:39</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>FAMILIA</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación de una nueva impresora en el puesto del solicitante, se hace la instalación respectiva y e l evidencia al solicitante el funcionamiento correcto de la impresora</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación de una nueva impresora en el puesto del solicitante, se hace la instalación respectiva y e l evidencia al solicitante el funcionamiento correcto de la impresora</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>6.	Apoyar en la documentación técnica del área, incluyendo la organización y archivo de documentos, informes de soporte y demás registros, de acuerdo con las directrices internas y del Sistema de Gestión de Calidad.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-03-11 08:16:56</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>OFICINA DE SISTEMAS</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ASESORIA Y ASISTENCIA</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Se solicita el acompañamiento de la capacitación del personal de Saimyr, se hace el acompañamiento respectivo y recolección de firmas necesario</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Se solicita el acompañamiento de la capacitación del personal de Saimyr, se hace el acompañamiento respectivo y recolección de firmas necesario</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-03-11 08:20:20</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ALMACEN MUNICIPAL</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Marcela</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación del escáner al equipo de la solicitante, se hace la instalación respectiva y se le evidencia a la solicitante el funcionamiento normal del escáner</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación del escáner al equipo de la solicitante, se hace la instalación respectiva y se le evidencia a la solicitante el funcionamiento normal del escáner</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2.	Apoyar en el mantenimiento preventivo básico de equipos tecnológicos, realizando tareas como limpieza, revisión de cables, conectores y periféricos, con el objetivo de mantener en condiciones óptimas los recursos informáticos de la entidad.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-03-11 08:22:25</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ALMACEN MUNICIPAL</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO PREVENTIVO</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Se solicita la eliminación de las impresoras que están instaladas en el equipo pero ya no se encuentran, se hace la eliminación respectiva y se le evidencia al funcionario</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Se solicita la eliminación de las impresoras que están instaladas en el equipo pero ya no se encuentran, se hace la eliminación respectiva y se le evidencia al funcionario</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>4.	Apoyar en tareas logísticas relacionadas con la infraestructura tecnológica, tales como instalación, traslado o reubicación de equipos de cómputo, dispositivos de red y demás componentes tecnológicos, bajo supervisión del personal del área.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-03-12 08:33:18</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>OFICINA DE SISTEMAS</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Mario Henao</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Se solicita el traslado de equipos dados de baja a los inservibles, se hace el traslado respectivo de estos equipos</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Se solicita el traslado de equipos dados de baja a los inservibles, se hace el traslado respectivo de estos equipos</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-03-12 08:39:22</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Elizabeth</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ASESORIA Y ASISTENCIA</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos de fiscales a los funcionarios, se hace la solicitud de permisos al encargado del modulo de ejecuciones fiscales se asignan los permisos solicitados</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos de fiscales a los funcionarios, se hace la solicitud de permisos al encargado del modulo de ejecuciones fiscales se asignan los permisos solicitados</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-03-13 08:52:39</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BIBLIOTECAS</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Saudith</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ASESORIA Y ASISTENCIA</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Se solicita la revisión y acompañamiento el personal de Tigo, se acompaña y se revisa y se plantea un cambio de equipo desde el técnico de Tigo</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Se solicita la revisión y acompañamiento el personal de Tigo, se acompaña y se revisa y se plantea un cambio de equipo desde el técnico de Tigo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-03-13 08:57:31</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EJECUCIONES FISCALES</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Se solicita la creación de un nuevo usuario para un nuevo funcionario en la dependencia, se hace la solicitud respectiva a los encargados de la plataforma Saimyr, se informa del nuevo usuario al solicitante</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Se solicita la creación de un nuevo usuario para un nuevo funcionario en la dependencia, se hace la solicitud respectiva a los encargados de la plataforma Saimyr, se informa del nuevo usuario al solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-03-16 11:11:55</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>BIBLIOTECAS</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Saudith</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ASESORIA Y ASISTENCIA</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Se solicita el acompañamiento en el cambio de equipo que estaba presentando el problema de interrupciones en el servicio de internet, se revisa que los servicios sigan funcionando</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Se solicita el acompañamiento en el cambio de equipo que estaba presentando el problema de interrupciones en el servicio de internet, se revisa que los servicios sigan funcionando</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>7.	Colaborar en la implementación y seguimiento de medidas básicas de seguridad informática, tales como el monitoreo de alertas básicas, cierre adecuado de sesiones, y cumplimiento de rutinas establecidas para el uso seguro de los recursos tecnológicos.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-03-16 11:25:03</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EJECUCIONES FISCALES</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Jarol</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Se solicita cambio de contraseña de acceso al modulo del solicitante, se hace el cambio solicitado y se le informa al solicitante</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Se solicita cambio de contraseña de acceso al modulo del solicitante, se hace el cambio solicitado y se le informa al solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-03-16 11:36:51</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EJECUCIONES FISCALES</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos al usuario solicitado, se asignan los permisos solicitados y se le informa al solicitante</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos al usuario solicitado, se asignan los permisos solicitados y se le informa al solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-03-23 11:56:35</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Elizabeth</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Se solicita la inhabilitación de módulos y eliminación de usuario para un funcionario que ya no se encuentra en la dependencia</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Se solicita la inhabilitación de módulos y eliminación de usuario para un funcionario que ya no se encuentra en la dependencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-03-17 17:18:30</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PLANEACIÓN</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Maribel</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO CORRECTIVE</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>LLAMADA TELEFONICA</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Se solicita la revisión de la impresora ya que esta salía una linea en el medio, se hace la revisión y limpieza respectiva y se le evidencia a la solicitante el funcionamiento normal de la impresora</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Se solicita la revisión de la impresora ya que esta salía una linea en el medio, se hace la revisión y limpieza respectiva y se le evidencia a la solicitante el funcionamiento normal de la impresora</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-03-17 17:21:20</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>PLANEACIÓN</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Juan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>MANTENIMIENTO CORRECTIVE</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Se solicita la revisión de la impresora pues salía un fallo al imprimir, se instala el driver correspondiente de la impresora y se evidencia el correcto funcionamiento de la impresora</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Se solicita la revisión de la impresora pues salía un fallo al imprimir, se instala el driver correspondiente de la impresora y se evidencia el correcto funcionamiento de la impresora</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-03-18 13:54:04</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Elizabeth</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Se solicita retirar los permisos en los módulos a funcionarios que ya no están en la administración o en la oficina de impuestos</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Se solicita retirar los permisos en los módulos a funcionarios que ya no están en la administración o en la oficina de impuestos</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>6.	Apoyar en la documentación técnica del área, incluyendo la organización y archivo de documentos, informes de soporte y demás registros, de acuerdo con las directrices internas y del Sistema de Gestión de Calidad.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-03-18 13:57:12</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>FAMILIA</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Luis Alejandro</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Configuración</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Descripcion de prueba - OK</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Prueba de observaciones - Subagent</t>
         </is>
       </c>
     </row>

</xml_diff>